<commit_message>
ADD: transport data for august
</commit_message>
<xml_diff>
--- a/transport/transport_data.xlsx
+++ b/transport/transport_data.xlsx
@@ -20912,16 +20912,16 @@
         </is>
       </c>
       <c r="J227" s="2" t="n">
-        <v>150</v>
+        <v>170</v>
       </c>
       <c r="K227" s="2" t="n">
         <v>15000</v>
       </c>
       <c r="L227" s="2" t="n">
-        <v>150</v>
+        <v>170</v>
       </c>
       <c r="M227" s="3" t="n">
-        <v>10</v>
+        <v>11.33333333333333</v>
       </c>
       <c r="O227" t="inlineStr">
         <is>
@@ -20945,7 +20945,7 @@
         </is>
       </c>
       <c r="W227" s="4" t="n">
-        <v>46230.74683976852</v>
+        <v>46237.71828126157</v>
       </c>
       <c r="X227" t="inlineStr">
         <is>
@@ -23775,6 +23775,4768 @@
       <c r="Z257" t="inlineStr">
         <is>
           <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="258" ht="19.2" customHeight="1">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>20260806-0001</t>
+        </is>
+      </c>
+      <c r="B258" s="1" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Варна-Бяла-Варна</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>Р2530ЕЕ</t>
+        </is>
+      </c>
+      <c r="J258" s="2" t="n">
+        <v>420</v>
+      </c>
+      <c r="K258" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L258" s="2" t="n">
+        <v>504</v>
+      </c>
+      <c r="M258" s="3" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="O258" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T258" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U258" s="4" t="n">
+        <v>46240.73343105324</v>
+      </c>
+      <c r="V258" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W258" s="4" t="n">
+        <v>46240.73788818287</v>
+      </c>
+      <c r="X258" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y258" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z258" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+    </row>
+    <row r="259" ht="19.2" customHeight="1">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>20260806-0002</t>
+        </is>
+      </c>
+      <c r="B259" s="1" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Бяла-Русе-Тервел-Гешаново-Близнаци-Русе</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>ДАНИЕЛ ПЕНЧЕВ ПЕНЧЕВ</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>Р7826КН</t>
+        </is>
+      </c>
+      <c r="J259" s="2" t="n">
+        <v>440</v>
+      </c>
+      <c r="K259" s="2" t="n">
+        <v>31000</v>
+      </c>
+      <c r="L259" s="2" t="n">
+        <v>528</v>
+      </c>
+      <c r="M259" s="3" t="n">
+        <v>17.03225806451613</v>
+      </c>
+      <c r="O259" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P259" s="2" t="n">
+        <v>31000</v>
+      </c>
+      <c r="T259" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U259" s="4" t="n">
+        <v>46240.73796966435</v>
+      </c>
+      <c r="V259" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W259" s="4" t="n">
+        <v>46240.73968159722</v>
+      </c>
+      <c r="X259" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y259" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z259" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+    </row>
+    <row r="260" ht="19.2" customHeight="1">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>20260806-0003</t>
+        </is>
+      </c>
+      <c r="B260" s="1" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Бяла-Русе-Варна-Добрич-Русе</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>ПАВЕЛ СТЕФАНОВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>CB2201CC</t>
+        </is>
+      </c>
+      <c r="J260" s="2" t="n">
+        <v>570</v>
+      </c>
+      <c r="K260" s="2" t="n">
+        <v>34000</v>
+      </c>
+      <c r="L260" s="2" t="n">
+        <v>684</v>
+      </c>
+      <c r="M260" s="3" t="n">
+        <v>20.11764705882353</v>
+      </c>
+      <c r="O260" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P260" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="T260" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U260" s="4" t="n">
+        <v>46240.73971719907</v>
+      </c>
+      <c r="V260" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W260" s="4" t="n">
+        <v>46240.74147510417</v>
+      </c>
+      <c r="X260" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y260" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z260" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+    </row>
+    <row r="261" ht="19.2" customHeight="1">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>20260806-0004</t>
+        </is>
+      </c>
+      <c r="B261" s="1" t="n">
+        <v>46240</v>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Варна-НХК-Каварна-Добрич-Повеляново-Терем-Варна</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>Р2530ЕЕ</t>
+        </is>
+      </c>
+      <c r="J261" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="K261" s="2" t="n">
+        <v>31000</v>
+      </c>
+      <c r="L261" s="2" t="n">
+        <v>600</v>
+      </c>
+      <c r="M261" s="3" t="n">
+        <v>19.35483870967742</v>
+      </c>
+      <c r="N261" s="2" t="n">
+        <v>15000</v>
+      </c>
+      <c r="O261" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P261" s="2" t="n">
+        <v>23000</v>
+      </c>
+      <c r="T261" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U261" s="4" t="n">
+        <v>46240.74150913194</v>
+      </c>
+      <c r="V261" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W261" s="4" t="n">
+        <v>46240.7443197338</v>
+      </c>
+      <c r="X261" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y261" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z261" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+    </row>
+    <row r="262" ht="19.2" customHeight="1">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>20260806-0005</t>
+        </is>
+      </c>
+      <c r="B262" s="1" t="n">
+        <v>46239</v>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Бяла-Русе-Нова камена-Тервел-Карапелит-Русе</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>ДАНИЕЛ ПЕНЧЕВ ПЕНЧЕВ</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>Р7826КН</t>
+        </is>
+      </c>
+      <c r="J262" s="2" t="n">
+        <v>430</v>
+      </c>
+      <c r="K262" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="L262" s="2" t="n">
+        <v>516</v>
+      </c>
+      <c r="M262" s="3" t="n">
+        <v>16.125</v>
+      </c>
+      <c r="O262" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P262" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="T262" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U262" s="4" t="n">
+        <v>46240.74437995371</v>
+      </c>
+      <c r="V262" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W262" s="4" t="n">
+        <v>46240.74647008102</v>
+      </c>
+      <c r="X262" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y262" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z262" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+    </row>
+    <row r="263" ht="19.2" customHeight="1">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>20260806-0006</t>
+        </is>
+      </c>
+      <c r="B263" s="1" t="n">
+        <v>46239</v>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Аспарухово-Бяла-Шумен-Вълчи дол-Добрич-Варна</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>"СИ-ТРАНС БЪЛГАРИЯ"  ЕООД</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>Живко Демиров Вълчев</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>В9261РА</t>
+        </is>
+      </c>
+      <c r="J263" s="2" t="n">
+        <v>485</v>
+      </c>
+      <c r="K263" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L263" s="2" t="n">
+        <v>510</v>
+      </c>
+      <c r="M263" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="O263" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P263" s="2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="T263" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U263" s="4" t="n">
+        <v>46240.74650496527</v>
+      </c>
+      <c r="V263" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W263" s="4" t="n">
+        <v>46241.46184988426</v>
+      </c>
+      <c r="X263" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y263" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z263" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+    </row>
+    <row r="264" ht="19.2" customHeight="1">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>20260806-0007</t>
+        </is>
+      </c>
+      <c r="B264" s="1" t="n">
+        <v>46239</v>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Варна-Девня-Повеляново-Осем ви-Аспарухово-Варна</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>Р2530ЕЕ</t>
+        </is>
+      </c>
+      <c r="J264" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="K264" s="2" t="n">
+        <v>26000</v>
+      </c>
+      <c r="L264" s="2" t="n">
+        <v>240</v>
+      </c>
+      <c r="M264" s="3" t="n">
+        <v>9.230769230769232</v>
+      </c>
+      <c r="N264" s="2" t="n">
+        <v>10000</v>
+      </c>
+      <c r="O264" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P264" s="2" t="n">
+        <v>29000</v>
+      </c>
+      <c r="T264" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U264" s="4" t="n">
+        <v>46240.75203077546</v>
+      </c>
+      <c r="V264" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W264" s="4" t="n">
+        <v>46240.75517672454</v>
+      </c>
+      <c r="X264" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y264" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z264" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+    </row>
+    <row r="265" ht="19.2" customHeight="1">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>20260806-0008</t>
+        </is>
+      </c>
+      <c r="B265" s="1" t="n">
+        <v>46239</v>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Русе-бяла-Пчелник-Варна</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>ПАВЕЛ СТЕФАНОВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>CB2201CC</t>
+        </is>
+      </c>
+      <c r="J265" s="2" t="n">
+        <v>290</v>
+      </c>
+      <c r="K265" s="2" t="n">
+        <v>16000</v>
+      </c>
+      <c r="L265" s="2" t="n">
+        <v>348</v>
+      </c>
+      <c r="M265" s="3" t="n">
+        <v>21.75</v>
+      </c>
+      <c r="O265" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T265" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U265" s="4" t="n">
+        <v>46240.7552682176</v>
+      </c>
+      <c r="V265" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W265" s="4" t="n">
+        <v>46240.75634476852</v>
+      </c>
+      <c r="X265" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y265" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z265" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+    </row>
+    <row r="266" ht="19.2" customHeight="1">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>20260806-0009</t>
+        </is>
+      </c>
+      <c r="B266" s="1" t="n">
+        <v>46238</v>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Варна-НХК-Каварна-Малина-Гешаново-Добрич-Варна</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>Р2530ЕЕ</t>
+        </is>
+      </c>
+      <c r="J266" s="2" t="n">
+        <v>480</v>
+      </c>
+      <c r="K266" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="L266" s="2" t="n">
+        <v>576</v>
+      </c>
+      <c r="M266" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="N266" s="2" t="n">
+        <v>21000</v>
+      </c>
+      <c r="O266" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P266" s="2" t="n">
+        <v>24000</v>
+      </c>
+      <c r="T266" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U266" s="4" t="n">
+        <v>46240.7564490625</v>
+      </c>
+      <c r="V266" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W266" s="4" t="n">
+        <v>46240.75857275463</v>
+      </c>
+      <c r="X266" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y266" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z266" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+    </row>
+    <row r="267" ht="19.2" customHeight="1">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>20260806-0010</t>
+        </is>
+      </c>
+      <c r="B267" s="1" t="n">
+        <v>46238</v>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>НХК-Чайка-Астер-Калина-Арсена-НХК</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>ДИРОСИ ООД</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>СТАНИСЛАВ ДИМИТРОВ ИВАНОВ</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>А1535ВВ</t>
+        </is>
+      </c>
+      <c r="J267" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="K267" s="2" t="n">
+        <v>6500</v>
+      </c>
+      <c r="L267" s="2" t="n">
+        <v>135</v>
+      </c>
+      <c r="M267" s="3" t="n">
+        <v>20.76923076923077</v>
+      </c>
+      <c r="O267" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T267" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U267" s="4" t="n">
+        <v>46240.75861923611</v>
+      </c>
+      <c r="V267" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W267" s="4" t="n">
+        <v>46240.7596140625</v>
+      </c>
+      <c r="X267" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y267" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z267" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+    </row>
+    <row r="268" ht="19.2" customHeight="1">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>20260806-0011</t>
+        </is>
+      </c>
+      <c r="B268" s="1" t="n">
+        <v>46238</v>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>НХК-Ден-Деветак-Съно-НХК</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>ДИРОСИ ООД</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>СТАНИСЛАВ ДИМИТРОВ ИВАНОВ</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>А1535ВВ</t>
+        </is>
+      </c>
+      <c r="J268" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="K268" s="2" t="n">
+        <v>13000</v>
+      </c>
+      <c r="L268" s="2" t="n">
+        <v>136</v>
+      </c>
+      <c r="M268" s="3" t="n">
+        <v>10.46153846153846</v>
+      </c>
+      <c r="O268" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P268" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="T268" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U268" s="4" t="n">
+        <v>46240.75967954861</v>
+      </c>
+      <c r="V268" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W268" s="4" t="n">
+        <v>46240.76422670139</v>
+      </c>
+      <c r="X268" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y268" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z268" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+    </row>
+    <row r="269" ht="19.2" customHeight="1">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>20260806-0012</t>
+        </is>
+      </c>
+      <c r="B269" s="1" t="n">
+        <v>46241</v>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>НХК-Чайка-НХК</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>РОСБУЛ ТРАНС</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>Милен Иванов Атанасов</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>А1535ВВ</t>
+        </is>
+      </c>
+      <c r="J269" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="K269" s="2" t="n">
+        <v>1500</v>
+      </c>
+      <c r="L269" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="M269" s="3" t="n">
+        <v>56.66666666666666</v>
+      </c>
+      <c r="O269" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T269" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U269" s="4" t="n">
+        <v>46240.76065498843</v>
+      </c>
+      <c r="V269" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W269" s="4" t="n">
+        <v>46240.7617344213</v>
+      </c>
+      <c r="X269" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y269" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z269" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+    </row>
+    <row r="270" ht="19.2" customHeight="1">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>20260806-0013</t>
+        </is>
+      </c>
+      <c r="B270" s="1" t="n">
+        <v>46237</v>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Варна-Аспарухово-Тервел-Гешаново-Добрич-Варна</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>ТРАНС ОЙЛ ЕООД</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>ДИАН СТОЯНОВ АЛЕКСАНДРОВ</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>B7902TM</t>
+        </is>
+      </c>
+      <c r="J270" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="K270" s="2" t="n">
+        <v>18000</v>
+      </c>
+      <c r="L270" s="2" t="n">
+        <v>3000</v>
+      </c>
+      <c r="M270" s="3" t="n">
+        <v>166.6666666666667</v>
+      </c>
+      <c r="O270" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P270" s="2" t="n">
+        <v>10000</v>
+      </c>
+      <c r="T270" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U270" s="4" t="n">
+        <v>46240.76179599537</v>
+      </c>
+      <c r="V270" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W270" s="4" t="n">
+        <v>46240.76312576389</v>
+      </c>
+      <c r="X270" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y270" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z270" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+    </row>
+    <row r="271" ht="19.2" customHeight="1">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>20260806-0014</t>
+        </is>
+      </c>
+      <c r="B271" s="1" t="n">
+        <v>46244</v>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Варна-Аспарухово-Добрич-Варна</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>Р2530ЕЕ</t>
+        </is>
+      </c>
+      <c r="J271" s="2" t="n">
+        <v>260</v>
+      </c>
+      <c r="K271" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L271" s="2" t="n">
+        <v>312</v>
+      </c>
+      <c r="M271" s="3" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="O271" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P271" s="2" t="n">
+        <v>14000</v>
+      </c>
+      <c r="T271" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U271" s="4" t="n">
+        <v>46240.76433942129</v>
+      </c>
+      <c r="V271" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W271" s="4" t="n">
+        <v>46244.64200315972</v>
+      </c>
+      <c r="X271" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y271" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z271" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+    </row>
+    <row r="272" ht="19.2" customHeight="1">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>20260810-0001</t>
+        </is>
+      </c>
+      <c r="B272" s="1" t="n">
+        <v>46245</v>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Русе-Бяла-Енево-Тервел-Русе</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>ДАНИЕЛ ПЕНЧЕВ ПЕНЧЕВ</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>Р7826КН</t>
+        </is>
+      </c>
+      <c r="J272" s="2" t="n">
+        <v>420</v>
+      </c>
+      <c r="K272" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="L272" s="2" t="n">
+        <v>504</v>
+      </c>
+      <c r="M272" s="3" t="n">
+        <v>15.75</v>
+      </c>
+      <c r="O272" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P272" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="T272" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U272" s="4" t="n">
+        <v>46244.64204703704</v>
+      </c>
+      <c r="V272" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W272" s="4" t="n">
+        <v>46244.64334456019</v>
+      </c>
+      <c r="X272" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y272" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z272" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="273" ht="19.2" customHeight="1">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>20260810-0002</t>
+        </is>
+      </c>
+      <c r="B273" s="1" t="n">
+        <v>46245</v>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Варна-нхк-Каварна-Добрич-Варна</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>Р2530ЕЕ</t>
+        </is>
+      </c>
+      <c r="J273" s="2" t="n">
+        <v>450</v>
+      </c>
+      <c r="K273" s="2" t="n">
+        <v>31000</v>
+      </c>
+      <c r="L273" s="2" t="n">
+        <v>540</v>
+      </c>
+      <c r="M273" s="3" t="n">
+        <v>17.41935483870968</v>
+      </c>
+      <c r="N273" s="2" t="n">
+        <v>18500</v>
+      </c>
+      <c r="O273" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P273" s="2" t="n">
+        <v>18500</v>
+      </c>
+      <c r="T273" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U273" s="4" t="n">
+        <v>46244.64341319445</v>
+      </c>
+      <c r="V273" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W273" s="4" t="n">
+        <v>46244.64645126157</v>
+      </c>
+      <c r="X273" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y273" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z273" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="274" ht="19.2" customHeight="1">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>20260810-0003</t>
+        </is>
+      </c>
+      <c r="B274" s="1" t="n">
+        <v>46245</v>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>НХК-Чайка хотел- НХК</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>РОСБУЛ ТРАНС</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>МИЛЕН СТЕФАНОВ АНДРЕЕВ</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>А2106НР</t>
+        </is>
+      </c>
+      <c r="J274" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="K274" s="2" t="n">
+        <v>1500</v>
+      </c>
+      <c r="L274" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="M274" s="3" t="n">
+        <v>56.66666666666666</v>
+      </c>
+      <c r="O274" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T274" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U274" s="4" t="n">
+        <v>46244.64656255787</v>
+      </c>
+      <c r="V274" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W274" s="4" t="n">
+        <v>46244.64750273148</v>
+      </c>
+      <c r="X274" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y274" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z274" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="275" ht="19.2" customHeight="1">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>20260810-0004</t>
+        </is>
+      </c>
+      <c r="B275" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>Варна-Аспарухово-Добрич-Варна</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>Р2530ЕЕ</t>
+        </is>
+      </c>
+      <c r="J275" s="2" t="n">
+        <v>260</v>
+      </c>
+      <c r="K275" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="L275" s="2" t="n">
+        <v>312</v>
+      </c>
+      <c r="M275" s="3" t="n">
+        <v>9.75</v>
+      </c>
+      <c r="O275" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P275" s="2" t="n">
+        <v>15600</v>
+      </c>
+      <c r="T275" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U275" s="4" t="n">
+        <v>46244.64761892361</v>
+      </c>
+      <c r="V275" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W275" s="4" t="n">
+        <v>46247.32354059027</v>
+      </c>
+      <c r="X275" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y275" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z275" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="276" ht="19.2" customHeight="1">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>20260810-0005</t>
+        </is>
+      </c>
+      <c r="B276" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Варна-Хидро-Варна</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>Р2530ЕЕ</t>
+        </is>
+      </c>
+      <c r="J276" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="K276" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="L276" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="M276" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="O276" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P276" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="T276" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U276" s="4" t="n">
+        <v>46244.64932045139</v>
+      </c>
+      <c r="V276" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W276" s="4" t="n">
+        <v>46247.32307840278</v>
+      </c>
+      <c r="X276" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y276" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z276" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+    </row>
+    <row r="277" ht="19.2" customHeight="1">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>20260813-0001</t>
+        </is>
+      </c>
+      <c r="B277" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Русе-Мечка-Русе</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>ЕЛ-ПЛАМ ТРАНС ЕООД</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>ЕЛКО ИВАНОВ ИВАНОВ</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>СВ5456СМ</t>
+        </is>
+      </c>
+      <c r="J277" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="K277" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L277" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="M277" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="O277" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P277" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="T277" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U277" s="4" t="n">
+        <v>46247.32360550926</v>
+      </c>
+      <c r="V277" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W277" s="4" t="n">
+        <v>46247.32470684028</v>
+      </c>
+      <c r="X277" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y277" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z277" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+    </row>
+    <row r="278" ht="19.2" customHeight="1">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>20260813-0002</t>
+        </is>
+      </c>
+      <c r="B278" s="1" t="n">
+        <v>46246</v>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>НХк-Община Поморие-НХК</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>ДЪЛВАН ЕООД</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>ИВАН ГЕОРГИЕВ ТУРМАНОВ</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>А7660КР</t>
+        </is>
+      </c>
+      <c r="J278" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="K278" s="2" t="n">
+        <v>8000</v>
+      </c>
+      <c r="L278" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="M278" s="3" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="O278" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P278" s="2" t="n">
+        <v>8000</v>
+      </c>
+      <c r="T278" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U278" s="4" t="n">
+        <v>46247.3248256713</v>
+      </c>
+      <c r="V278" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W278" s="4" t="n">
+        <v>46247.32540394676</v>
+      </c>
+      <c r="X278" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y278" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z278" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+    </row>
+    <row r="279" ht="19.2" customHeight="1">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>20260813-0003</t>
+        </is>
+      </c>
+      <c r="B279" s="1" t="n">
+        <v>46247</v>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Варна-НХК-Каварна-Шабла-Добрич-Варна</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>Р2530ЕЕ</t>
+        </is>
+      </c>
+      <c r="J279" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="K279" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L279" s="2" t="n">
+        <v>600</v>
+      </c>
+      <c r="M279" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="N279" s="2" t="n">
+        <v>15000</v>
+      </c>
+      <c r="O279" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P279" s="2" t="n">
+        <v>15000</v>
+      </c>
+      <c r="T279" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U279" s="4" t="n">
+        <v>46247.32544461806</v>
+      </c>
+      <c r="V279" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W279" s="4" t="n">
+        <v>46247.33645689815</v>
+      </c>
+      <c r="X279" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y279" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z279" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+    </row>
+    <row r="280" ht="19.2" customHeight="1">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>20260813-0004</t>
+        </is>
+      </c>
+      <c r="B280" s="1" t="n">
+        <v>46247</v>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Варна-Малина-Добрич-Варна</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>ТРАНС ОЙЛ ЕООД</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>ДИАН СТОЯНОВ АЛЕКСАНДРОВ</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>B7902TM</t>
+        </is>
+      </c>
+      <c r="J280" s="2" t="n">
+        <v>135</v>
+      </c>
+      <c r="K280" s="2" t="n">
+        <v>12000</v>
+      </c>
+      <c r="L280" s="2" t="n">
+        <v>135</v>
+      </c>
+      <c r="M280" s="3" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="O280" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P280" s="2" t="n">
+        <v>4000</v>
+      </c>
+      <c r="T280" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U280" s="4" t="n">
+        <v>46247.3364921875</v>
+      </c>
+      <c r="V280" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W280" s="4" t="n">
+        <v>46247.42416609954</v>
+      </c>
+      <c r="X280" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y280" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z280" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+    </row>
+    <row r="281" ht="19.2" customHeight="1">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>20260813-0005</t>
+        </is>
+      </c>
+      <c r="B281" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Варна-Добрич-Варна</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>ТРАНС ОЙЛ ЕООД</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>ДИАН СТОЯНОВ АЛЕКСАНДРОВ</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>B7902TM</t>
+        </is>
+      </c>
+      <c r="J281" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="K281" s="2" t="n">
+        <v>16000</v>
+      </c>
+      <c r="L281" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="M281" s="3" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="O281" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T281" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U281" s="4" t="n">
+        <v>46247.42525802083</v>
+      </c>
+      <c r="V281" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W281" s="4" t="n">
+        <v>46247.42672533564</v>
+      </c>
+      <c r="X281" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y281" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z281" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+    </row>
+    <row r="282" ht="19.2" customHeight="1">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>20260813-0006</t>
+        </is>
+      </c>
+      <c r="B282" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Русе-Тервел-Нова Камена-Карапелит-Русе</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>ДАНИЕЛ ПЕНЧЕВ ПЕНЧЕВ</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>Р7826КН</t>
+        </is>
+      </c>
+      <c r="J282" s="2" t="n">
+        <v>390</v>
+      </c>
+      <c r="K282" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="L282" s="2" t="n">
+        <v>468</v>
+      </c>
+      <c r="M282" s="3" t="n">
+        <v>14.625</v>
+      </c>
+      <c r="O282" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P282" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="T282" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U282" s="4" t="n">
+        <v>46247.42680295139</v>
+      </c>
+      <c r="V282" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W282" s="4" t="n">
+        <v>46247.42994275463</v>
+      </c>
+      <c r="X282" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y282" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z282" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+    </row>
+    <row r="283" ht="19.2" customHeight="1">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>20260813-0007</t>
+        </is>
+      </c>
+      <c r="B283" s="1" t="n">
+        <v>46248</v>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Варна-Аспарухово-Дългопол-Брестак-Киселово-Варна</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>Р2530ЕЕ</t>
+        </is>
+      </c>
+      <c r="J283" s="2" t="n">
+        <v>230</v>
+      </c>
+      <c r="K283" s="2" t="n">
+        <v>35000</v>
+      </c>
+      <c r="L283" s="2" t="n">
+        <v>276</v>
+      </c>
+      <c r="M283" s="3" t="n">
+        <v>7.885714285714286</v>
+      </c>
+      <c r="O283" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P283" s="2" t="n">
+        <v>35000</v>
+      </c>
+      <c r="T283" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U283" s="4" t="n">
+        <v>46247.42998789352</v>
+      </c>
+      <c r="V283" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W283" s="4" t="n">
+        <v>46247.43157589121</v>
+      </c>
+      <c r="X283" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y283" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z283" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+    </row>
+    <row r="284" ht="19.2" customHeight="1">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>20260819-0001</t>
+        </is>
+      </c>
+      <c r="B284" s="1" t="n">
+        <v>46251</v>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Варна-Бомби-КРЗ-Братя-Салс-Киров-Варна</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>Р2530ЕЕ</t>
+        </is>
+      </c>
+      <c r="J284" s="2" t="n">
+        <v>320</v>
+      </c>
+      <c r="K284" s="2" t="n">
+        <v>36400</v>
+      </c>
+      <c r="L284" s="2" t="n">
+        <v>384</v>
+      </c>
+      <c r="M284" s="3" t="n">
+        <v>10.54945054945055</v>
+      </c>
+      <c r="N284" s="2" t="n">
+        <v>12000</v>
+      </c>
+      <c r="O284" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P284" s="2" t="n">
+        <v>26400</v>
+      </c>
+      <c r="T284" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U284" s="4" t="n">
+        <v>46253.44973041667</v>
+      </c>
+      <c r="V284" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W284" s="4" t="n">
+        <v>46253.45206186343</v>
+      </c>
+      <c r="X284" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y284" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z284" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="285" ht="19.2" customHeight="1">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>20260819-0002</t>
+        </is>
+      </c>
+      <c r="B285" s="1" t="n">
+        <v>46252</v>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Варна-Аспарухово-Добрич-Варна</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>Р2530ЕЕ</t>
+        </is>
+      </c>
+      <c r="J285" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="K285" s="2" t="n">
+        <v>28300</v>
+      </c>
+      <c r="L285" s="2" t="n">
+        <v>336</v>
+      </c>
+      <c r="M285" s="3" t="n">
+        <v>11.87279151943463</v>
+      </c>
+      <c r="O285" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T285" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U285" s="4" t="n">
+        <v>46253.45210194444</v>
+      </c>
+      <c r="V285" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W285" s="4" t="n">
+        <v>46253.45332358796</v>
+      </c>
+      <c r="X285" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y285" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z285" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="286" ht="19.2" customHeight="1">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>20260819-0003</t>
+        </is>
+      </c>
+      <c r="B286" s="1" t="n">
+        <v>46252</v>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Варна-Ген.Тошево-Сенокос-Варна</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>ТРАНС ОЙЛ ЕООД</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>ДИАН СТОЯНОВ АЛЕКСАНДРОВ</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>B7902TM</t>
+        </is>
+      </c>
+      <c r="J286" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="K286" s="2" t="n">
+        <v>18000</v>
+      </c>
+      <c r="L286" s="2" t="n">
+        <v>180</v>
+      </c>
+      <c r="M286" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="O286" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P286" s="2" t="n">
+        <v>14000</v>
+      </c>
+      <c r="T286" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U286" s="4" t="n">
+        <v>46253.45335928241</v>
+      </c>
+      <c r="V286" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W286" s="4" t="n">
+        <v>46253.45457443287</v>
+      </c>
+      <c r="X286" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y286" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z286" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="287" ht="19.2" customHeight="1">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>20260819-0004</t>
+        </is>
+      </c>
+      <c r="B287" s="1" t="n">
+        <v>46252</v>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Русе-Снежина-Русе</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>АЛМА ТРАНС ЕООД</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>Теодор Александров Георгиев</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>ОВ7977ВА</t>
+        </is>
+      </c>
+      <c r="J287" s="2" t="n">
+        <v>165</v>
+      </c>
+      <c r="K287" s="2" t="n">
+        <v>18700</v>
+      </c>
+      <c r="L287" s="2" t="n">
+        <v>281</v>
+      </c>
+      <c r="M287" s="3" t="n">
+        <v>15.02673796791444</v>
+      </c>
+      <c r="O287" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P287" s="2" t="n">
+        <v>18700</v>
+      </c>
+      <c r="T287" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U287" s="4" t="n">
+        <v>46253.45460394676</v>
+      </c>
+      <c r="V287" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W287" s="4" t="n">
+        <v>46253.47334265046</v>
+      </c>
+      <c r="X287" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y287" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z287" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="288" ht="19.2" customHeight="1">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>20260819-0005</t>
+        </is>
+      </c>
+      <c r="B288" s="1" t="n">
+        <v>46252</v>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Русе-Тервел-Кладенци-Жегларци-Русе</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>АЛМА ТРАНС ЕООД</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>Теодор Александров Георгиев</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>ОВ7977ВА</t>
+        </is>
+      </c>
+      <c r="J288" s="2" t="n">
+        <v>195</v>
+      </c>
+      <c r="K288" s="2" t="n">
+        <v>17500</v>
+      </c>
+      <c r="L288" s="2" t="n">
+        <v>331</v>
+      </c>
+      <c r="M288" s="3" t="n">
+        <v>18.91428571428571</v>
+      </c>
+      <c r="O288" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P288" s="2" t="n">
+        <v>17500</v>
+      </c>
+      <c r="T288" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U288" s="4" t="n">
+        <v>46253.47354578703</v>
+      </c>
+      <c r="V288" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W288" s="4" t="n">
+        <v>46253.47483068287</v>
+      </c>
+      <c r="X288" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y288" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z288" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="289" ht="19.2" customHeight="1">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>20260819-0006</t>
+        </is>
+      </c>
+      <c r="B289" s="1" t="n">
+        <v>46253</v>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>НХК-Каблешково-Слънчев бряг-НХК</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>РОСБУЛ ТРАНС</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>Милен Иванов Атанасов</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>А2106НР</t>
+        </is>
+      </c>
+      <c r="J289" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="K289" s="2" t="n">
+        <v>7800</v>
+      </c>
+      <c r="L289" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="M289" s="3" t="n">
+        <v>10.8974358974359</v>
+      </c>
+      <c r="O289" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P289" s="2" t="n">
+        <v>1800</v>
+      </c>
+      <c r="T289" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U289" s="4" t="n">
+        <v>46253.47493780093</v>
+      </c>
+      <c r="V289" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W289" s="4" t="n">
+        <v>46253.47946357639</v>
+      </c>
+      <c r="X289" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y289" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z289" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="290" ht="19.2" customHeight="1">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>20260819-0007</t>
+        </is>
+      </c>
+      <c r="B290" s="1" t="n">
+        <v>46253</v>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Варна-Аспарухово-Енево-Варна</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="J290" s="2" t="n">
+        <v>210</v>
+      </c>
+      <c r="K290" s="2" t="n">
+        <v>26200</v>
+      </c>
+      <c r="L290" s="2" t="n">
+        <v>252</v>
+      </c>
+      <c r="M290" s="3" t="n">
+        <v>9.618320610687023</v>
+      </c>
+      <c r="N290" s="2" t="n">
+        <v>11200</v>
+      </c>
+      <c r="O290" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P290" s="2" t="n">
+        <v>25200</v>
+      </c>
+      <c r="T290" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U290" s="4" t="n">
+        <v>46253.47952993056</v>
+      </c>
+      <c r="V290" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W290" s="4" t="n">
+        <v>46253.48405149305</v>
+      </c>
+      <c r="X290" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y290" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z290" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="291" ht="19.2" customHeight="1">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>20260819-0008</t>
+        </is>
+      </c>
+      <c r="B291" s="1" t="n">
+        <v>46253</v>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Варна-НХК-Пчелник-Девня-Добрич-Варна</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>"СИ-ТРАНС БЪЛГАРИЯ"  ЕООД</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>Живко Демиров Вълчев</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>В9261РА</t>
+        </is>
+      </c>
+      <c r="J291" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="K291" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L291" s="2" t="n">
+        <v>420</v>
+      </c>
+      <c r="M291" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="O291" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T291" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U291" s="4" t="n">
+        <v>46253.48409303241</v>
+      </c>
+      <c r="V291" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W291" s="4" t="n">
+        <v>46253.4856337963</v>
+      </c>
+      <c r="X291" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y291" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z291" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="292" ht="19.2" customHeight="1">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>20260819-0009</t>
+        </is>
+      </c>
+      <c r="B292" s="1" t="n">
+        <v>46254</v>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Русе-Тервел-Риш-Невестино-Деветак-НХК</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>ДАНИЕЛ ПЕНЧЕВ ПЕНЧЕВ</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>Р7826КН</t>
+        </is>
+      </c>
+      <c r="J292" s="2" t="n">
+        <v>440</v>
+      </c>
+      <c r="K292" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="L292" s="2" t="n">
+        <v>528</v>
+      </c>
+      <c r="M292" s="3" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="O292" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P292" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="T292" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U292" s="4" t="n">
+        <v>46253.4857122338</v>
+      </c>
+      <c r="V292" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W292" s="4" t="n">
+        <v>46258.70121236111</v>
+      </c>
+      <c r="X292" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y292" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z292" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+    </row>
+    <row r="293" ht="19.2" customHeight="1">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>20260824-0001</t>
+        </is>
+      </c>
+      <c r="B293" s="1" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Варна-Аспарухово-Варна-Добрич-Красен-Варна</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>ТРАНС ОЙЛ ЕООД</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>ДИАН СТОЯНОВ АЛЕКСАНДРОВ</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>B7902TM</t>
+        </is>
+      </c>
+      <c r="J293" s="2" t="n">
+        <v>330</v>
+      </c>
+      <c r="K293" s="2" t="n">
+        <v>18000</v>
+      </c>
+      <c r="L293" s="2" t="n">
+        <v>330</v>
+      </c>
+      <c r="M293" s="3" t="n">
+        <v>18.33333333333333</v>
+      </c>
+      <c r="O293" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P293" s="2" t="n">
+        <v>4000</v>
+      </c>
+      <c r="T293" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U293" s="4" t="n">
+        <v>46258.70141886574</v>
+      </c>
+      <c r="V293" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W293" s="4" t="n">
+        <v>46258.70329149305</v>
+      </c>
+      <c r="X293" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y293" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z293" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="294" ht="19.2" customHeight="1">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>20260824-0002</t>
+        </is>
+      </c>
+      <c r="B294" s="1" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Варна-Каварна-Добрич-Варна</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>ТРАНС ОЙЛ ЕООД</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>ДИАН СТОЯНОВ АЛЕКСАНДРОВ</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>B7902TM</t>
+        </is>
+      </c>
+      <c r="J294" s="2" t="n">
+        <v>190</v>
+      </c>
+      <c r="K294" s="2" t="n">
+        <v>18000</v>
+      </c>
+      <c r="L294" s="2" t="n">
+        <v>190</v>
+      </c>
+      <c r="M294" s="3" t="n">
+        <v>10.55555555555556</v>
+      </c>
+      <c r="O294" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P294" s="2" t="n">
+        <v>13000</v>
+      </c>
+      <c r="T294" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U294" s="4" t="n">
+        <v>46258.70332947917</v>
+      </c>
+      <c r="V294" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W294" s="4" t="n">
+        <v>46258.70728408565</v>
+      </c>
+      <c r="X294" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y294" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z294" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="295" ht="19.2" customHeight="1">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>20260824-0003</t>
+        </is>
+      </c>
+      <c r="B295" s="1" t="n">
+        <v>46255</v>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>НХК-Долни Чифлик - Каварна - Метличина - Карапелит - Житница - Тервел - Русе</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>ДАНИЕЛ ПЕНЧЕВ ПЕНЧЕВ</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>Р7826КН</t>
+        </is>
+      </c>
+      <c r="J295" s="2" t="n">
+        <v>590</v>
+      </c>
+      <c r="K295" s="2" t="n">
+        <v>32300</v>
+      </c>
+      <c r="L295" s="2" t="n">
+        <v>708</v>
+      </c>
+      <c r="M295" s="3" t="n">
+        <v>21.91950464396285</v>
+      </c>
+      <c r="O295" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P295" s="2" t="n">
+        <v>32300</v>
+      </c>
+      <c r="T295" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U295" s="4" t="n">
+        <v>46258.70732233796</v>
+      </c>
+      <c r="V295" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W295" s="4" t="n">
+        <v>46258.71006979167</v>
+      </c>
+      <c r="X295" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y295" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z295" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="296" ht="19.2" customHeight="1">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>20260824-0004</t>
+        </is>
+      </c>
+      <c r="B296" s="1" t="n">
+        <v>46258</v>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Варна-НХК-Пчелник-Каварна-Малина-Добрич-Варна</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>"СИ-ТРАНС БЪЛГАРИЯ"  ЕООД</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>Живко Демиров Вълчев</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>В9296ТМ</t>
+        </is>
+      </c>
+      <c r="J296" s="2" t="n">
+        <v>516</v>
+      </c>
+      <c r="K296" s="2" t="n">
+        <v>31000</v>
+      </c>
+      <c r="L296" s="2" t="n">
+        <v>550</v>
+      </c>
+      <c r="M296" s="3" t="n">
+        <v>17.74193548387097</v>
+      </c>
+      <c r="O296" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P296" s="2" t="n">
+        <v>22200</v>
+      </c>
+      <c r="T296" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U296" s="4" t="n">
+        <v>46258.71017533565</v>
+      </c>
+      <c r="V296" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W296" s="4" t="n">
+        <v>46259.43945784722</v>
+      </c>
+      <c r="X296" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y296" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z296" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="297" ht="19.2" customHeight="1">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>20260824-0005</t>
+        </is>
+      </c>
+      <c r="B297" s="1" t="n">
+        <v>46258</v>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Русе-Тервел-Брестак-Ген. Колево - Добрич -Аспарухово</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>ПАВЕЛ СТЕФАНОВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>CB2201CC</t>
+        </is>
+      </c>
+      <c r="J297" s="2" t="n">
+        <v>400</v>
+      </c>
+      <c r="K297" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="L297" s="2" t="n">
+        <v>480</v>
+      </c>
+      <c r="M297" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="O297" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P297" s="2" t="n">
+        <v>28000</v>
+      </c>
+      <c r="T297" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U297" s="4" t="n">
+        <v>46258.71245950231</v>
+      </c>
+      <c r="V297" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W297" s="4" t="n">
+        <v>46258.71662456018</v>
+      </c>
+      <c r="X297" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y297" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z297" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="298" ht="19.2" customHeight="1">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>20260825-0001</t>
+        </is>
+      </c>
+      <c r="B298" s="1" t="n">
+        <v>46259</v>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Салс-Салс</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>"СИ-ТРАНС БЪЛГАРИЯ"  ЕООД</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>Живко Демиров Вълчев</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>В9296ТМ</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>В6351ЕН</t>
+        </is>
+      </c>
+      <c r="K298" s="2" t="n">
+        <v>8500</v>
+      </c>
+      <c r="L298" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="M298" s="3" t="n">
+        <v>14.11764705882353</v>
+      </c>
+      <c r="O298" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P298" s="2" t="n">
+        <v>8500</v>
+      </c>
+      <c r="T298" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U298" s="4" t="n">
+        <v>46259.60008709491</v>
+      </c>
+      <c r="V298" t="inlineStr">
+        <is>
+          <t>Plamen Svetoslavov</t>
+        </is>
+      </c>
+      <c r="W298" s="4" t="n">
+        <v>46262.65285101852</v>
+      </c>
+      <c r="X298" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y298" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z298" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="299" ht="19.2" customHeight="1">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>20260825-0002</t>
+        </is>
+      </c>
+      <c r="B299" s="1" t="n">
+        <v>46260</v>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Русе-Бяла-Орешец</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>ЕЛ-ПЛАМ ТРАНС ЕООД</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>ТОДОР  ДИМИТРОВ ИВАНОВ</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>В9261РА</t>
+        </is>
+      </c>
+      <c r="J299" s="2" t="n">
+        <v>335</v>
+      </c>
+      <c r="K299" s="2" t="n">
+        <v>18700</v>
+      </c>
+      <c r="L299" s="2" t="n">
+        <v>570</v>
+      </c>
+      <c r="M299" s="3" t="n">
+        <v>30.48128342245989</v>
+      </c>
+      <c r="O299" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P299" s="2" t="n">
+        <v>18700</v>
+      </c>
+      <c r="T299" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U299" s="4" t="n">
+        <v>46259.60184413195</v>
+      </c>
+      <c r="V299" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W299" s="4" t="n">
+        <v>46259.60305853009</v>
+      </c>
+      <c r="X299" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y299" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z299" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="300" ht="19.2" customHeight="1">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>20260825-0003</t>
+        </is>
+      </c>
+      <c r="B300" s="1" t="n">
+        <v>46260</v>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>НХК-Калина Гадън-НХК</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>ДИРОСИ ООД</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>СТАНИСЛАВ ДИМИТРОВ ИВАНОВ</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>А1535ВВ</t>
+        </is>
+      </c>
+      <c r="K300" s="2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="L300" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="M300" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="O300" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="T300" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U300" s="4" t="n">
+        <v>46259.60308570602</v>
+      </c>
+      <c r="V300" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W300" s="4" t="n">
+        <v>46259.60364623843</v>
+      </c>
+      <c r="X300" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y300" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z300" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="301" ht="19.2" customHeight="1">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>20260825-0004</t>
+        </is>
+      </c>
+      <c r="B301" s="1" t="n">
+        <v>46260</v>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>Бяла-Добрич-Варна-НХК</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>ПАВЕЛ СТЕФАНОВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>Р9581МА</t>
+        </is>
+      </c>
+      <c r="J301" s="2" t="n">
+        <v>520</v>
+      </c>
+      <c r="K301" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L301" s="2" t="n">
+        <v>624</v>
+      </c>
+      <c r="M301" s="3" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="O301" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P301" s="2" t="n">
+        <v>15000</v>
+      </c>
+      <c r="T301" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U301" s="4" t="n">
+        <v>46259.60367255787</v>
+      </c>
+      <c r="V301" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W301" s="4" t="n">
+        <v>46259.60668869213</v>
+      </c>
+      <c r="X301" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y301" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z301" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="302" ht="19.2" customHeight="1">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>20260825-0005</t>
+        </is>
+      </c>
+      <c r="B302" s="1" t="n">
+        <v>46261</v>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>СЗ-Бяла-СЗ-Крепост-Димитровград-СЗ</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>ЗАРА Е</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>СТЕФАН ГОСПОДИНОВ СТАЛЕВ</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>СТ4211РА</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>СТ3099ЕН</t>
+        </is>
+      </c>
+      <c r="J302" s="2" t="n">
+        <v>451</v>
+      </c>
+      <c r="K302" s="2" t="n">
+        <v>31000</v>
+      </c>
+      <c r="L302" s="2" t="n">
+        <v>587</v>
+      </c>
+      <c r="M302" s="3" t="n">
+        <v>18.93548387096774</v>
+      </c>
+      <c r="O302" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P302" s="2" t="n">
+        <v>27000</v>
+      </c>
+      <c r="T302" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U302" s="4" t="n">
+        <v>46259.6091428588</v>
+      </c>
+      <c r="V302" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W302" s="4" t="n">
+        <v>46262.62206979167</v>
+      </c>
+      <c r="X302" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y302" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z302" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+    </row>
+    <row r="303" ht="19.2" customHeight="1">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>20260828-0001</t>
+        </is>
+      </c>
+      <c r="B303" s="1" t="n">
+        <v>46261</v>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Русе-Повеляново-Калиманци - Каварна-Русе</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>ПАВЕЛ СТЕФАНОВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>Р7826КН</t>
+        </is>
+      </c>
+      <c r="J303" s="2" t="n">
+        <v>520</v>
+      </c>
+      <c r="K303" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="L303" s="2" t="n">
+        <v>624</v>
+      </c>
+      <c r="M303" s="3" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="O303" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P303" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="T303" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U303" s="4" t="n">
+        <v>46262.62210945602</v>
+      </c>
+      <c r="V303" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W303" s="4" t="n">
+        <v>46262.62692824074</v>
+      </c>
+      <c r="X303" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y303" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z303" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="304" ht="19.2" customHeight="1">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>20260828-0002</t>
+        </is>
+      </c>
+      <c r="B304" s="1" t="n">
+        <v>46261</v>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Бяла-Русе-Северняк-Добрич-Варна-Русе</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>СДР Трайл ЕООД</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>РОМАН ЙОРДАНОВ ЗДРАВКОВ</t>
+        </is>
+      </c>
+      <c r="J304" s="2" t="n">
+        <v>550</v>
+      </c>
+      <c r="K304" s="2" t="n">
+        <v>30000</v>
+      </c>
+      <c r="L304" s="2" t="n">
+        <v>825</v>
+      </c>
+      <c r="M304" s="3" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="O304" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P304" s="2" t="n">
+        <v>2000</v>
+      </c>
+      <c r="T304" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U304" s="4" t="n">
+        <v>46262.62697130787</v>
+      </c>
+      <c r="V304" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W304" s="4" t="n">
+        <v>46262.62812802083</v>
+      </c>
+      <c r="X304" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y304" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z304" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="305" ht="19.2" customHeight="1">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>20260828-0003</t>
+        </is>
+      </c>
+      <c r="B305" s="1" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Бяла-Варна-Добрич-Русе</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>ПАВЕЛ СТЕФАНОВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="J305" s="2" t="n">
+        <v>470</v>
+      </c>
+      <c r="K305" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="L305" s="2" t="n">
+        <v>564</v>
+      </c>
+      <c r="M305" s="3" t="n">
+        <v>17.625</v>
+      </c>
+      <c r="O305" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P305" s="2" t="n">
+        <v>20000</v>
+      </c>
+      <c r="T305" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U305" s="4" t="n">
+        <v>46262.62816707176</v>
+      </c>
+      <c r="V305" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W305" s="4" t="n">
+        <v>46262.6311090625</v>
+      </c>
+      <c r="X305" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y305" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z305" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="306" ht="19.2" customHeight="1">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>20260828-0004</t>
+        </is>
+      </c>
+      <c r="B306" s="1" t="n">
+        <v>46262</v>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Бяла-Варна-Добрич-Тервел-Русе</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>ВЕНЦИСЛАВ КРУМОВ</t>
+        </is>
+      </c>
+      <c r="J306" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="K306" s="2" t="n">
+        <v>20000</v>
+      </c>
+      <c r="L306" s="2" t="n">
+        <v>550</v>
+      </c>
+      <c r="M306" s="3" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="O306" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P306" s="2" t="n">
+        <v>7000</v>
+      </c>
+      <c r="T306" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U306" s="4" t="n">
+        <v>46262.63115662037</v>
+      </c>
+      <c r="V306" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W306" s="4" t="n">
+        <v>46262.63226666667</v>
+      </c>
+      <c r="X306" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y306" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z306" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="307" ht="19.2" customHeight="1">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>20260828-0005</t>
+        </is>
+      </c>
+      <c r="B307" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Варна-НХК-Каварна-Добрич-Варна</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>ГЕОРГИ ИЛИЕВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="J307" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="K307" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="L307" s="2" t="n">
+        <v>600</v>
+      </c>
+      <c r="M307" s="3" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="N307" s="2" t="n">
+        <v>12000</v>
+      </c>
+      <c r="O307" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P307" s="2" t="n">
+        <v>16000</v>
+      </c>
+      <c r="T307" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U307" s="4" t="n">
+        <v>46262.63231280092</v>
+      </c>
+      <c r="V307" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W307" s="4" t="n">
+        <v>46262.63573277778</v>
+      </c>
+      <c r="X307" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y307" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z307" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="308" ht="19.2" customHeight="1">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>20260828-0006</t>
+        </is>
+      </c>
+      <c r="B308" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Русе-Тервел-Нова Камена - Гешаново-Русе</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>ЕВРОУЕЙ СЪРВИЗ ООД</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>ПАВЕЛ СТЕФАНОВ ГЕОРГИЕВ</t>
+        </is>
+      </c>
+      <c r="J308" s="2" t="n">
+        <v>440</v>
+      </c>
+      <c r="K308" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="L308" s="2" t="n">
+        <v>528</v>
+      </c>
+      <c r="M308" s="3" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="O308" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P308" s="2" t="n">
+        <v>32000</v>
+      </c>
+      <c r="T308" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U308" s="4" t="n">
+        <v>46262.63578925926</v>
+      </c>
+      <c r="V308" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W308" s="4" t="n">
+        <v>46262.63877578704</v>
+      </c>
+      <c r="X308" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y308" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z308" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+    </row>
+    <row r="309" ht="19.2" customHeight="1">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>20260831-0001</t>
+        </is>
+      </c>
+      <c r="B309" s="1" t="n">
+        <v>46265</v>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>ОФИС ВАРНА</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>НХК-Поморие</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>ДЪЛВАН ЕООД</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>ИВАН ГЕОРГИЕВ ТУРМАНОВ</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>А7660КР</t>
+        </is>
+      </c>
+      <c r="K309" s="2" t="n">
+        <v>8000</v>
+      </c>
+      <c r="M309" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O309" t="inlineStr">
+        <is>
+          <t>НЕПЛАТЕНА</t>
+        </is>
+      </c>
+      <c r="P309" s="2" t="n">
+        <v>8000</v>
+      </c>
+      <c r="T309" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="U309" s="4" t="n">
+        <v>46265.65786912037</v>
+      </c>
+      <c r="V309" t="inlineStr">
+        <is>
+          <t>Vesela Nikolova</t>
+        </is>
+      </c>
+      <c r="W309" s="4" t="n">
+        <v>46265.65914315972</v>
+      </c>
+      <c r="X309" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="Y309" t="inlineStr">
+        <is>
+          <t>08</t>
+        </is>
+      </c>
+      <c r="Z309" t="inlineStr">
+        <is>
+          <t>31</t>
         </is>
       </c>
     </row>

</xml_diff>